<commit_message>
Add 9_Date_Time_Functions & update Text_functions
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/8_Text_Functions.xlsx
+++ b/2_Formulas_Functions/8_Text_Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7456b23f02075ab8/Documents/Excel LUKE/2_Formulas_Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{B814E771-D0B5-4FE9-A208-226CFD245E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{495532FD-7CAC-4CAA-B29C-F77E81C3A969}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{B814E771-D0B5-4FE9-A208-226CFD245E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F605B35B-C4BD-4896-B5CF-E859E37DD42A}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{547B0A3B-DA78-41AD-863F-BF345DD25DB8}"/>
   </bookViews>
@@ -936,7 +936,7 @@
         <v>13</v>
       </c>
       <c r="V2" t="str">
-        <f>MID(G2,T2,2)</f>
+        <f>MID(G2,T2,U2-T2)</f>
         <v>CA</v>
       </c>
     </row>
@@ -993,6 +993,18 @@
         <f t="shared" ref="S3:S21" si="6">MID(G3,Q3,R3-Q3)</f>
         <v>IL</v>
       </c>
+      <c r="T3">
+        <f t="shared" ref="T3:T21" si="7">FIND(",",G3)+LEN(", ")</f>
+        <v>10</v>
+      </c>
+      <c r="U3">
+        <f t="shared" ref="U3:U21" si="8">FIND(",",G3,T3)</f>
+        <v>12</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V21" si="9">MID(G3,T3,U3-T3)</f>
+        <v>IL</v>
+      </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -1047,6 +1059,18 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T4">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U4">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1101,6 +1125,18 @@
         <f t="shared" si="6"/>
         <v>CA</v>
       </c>
+      <c r="T5">
+        <f t="shared" si="7"/>
+        <v>11</v>
+      </c>
+      <c r="U5">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="9"/>
+        <v>CA</v>
+      </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
@@ -1155,6 +1191,18 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T6">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -1209,6 +1257,18 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T7">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -1263,6 +1323,18 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T8">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
@@ -1317,6 +1389,18 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T9">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
@@ -1371,6 +1455,18 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T10">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
@@ -1425,6 +1521,18 @@
         <f t="shared" si="6"/>
         <v>CA</v>
       </c>
+      <c r="T11">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="8"/>
+        <v>16</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="9"/>
+        <v>CA</v>
+      </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -1479,6 +1587,18 @@
         <f t="shared" si="6"/>
         <v>CA</v>
       </c>
+      <c r="T12">
+        <f t="shared" si="7"/>
+        <v>12</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="8"/>
+        <v>14</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="9"/>
+        <v>CA</v>
+      </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
@@ -1533,6 +1653,18 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T13">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -1587,6 +1719,18 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T14">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
@@ -1641,6 +1785,18 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T15">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V15" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
@@ -1695,8 +1851,20 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T16">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V16" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>79</v>
       </c>
@@ -1749,8 +1917,20 @@
         <f t="shared" si="6"/>
         <v>IL</v>
       </c>
+      <c r="T17">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="8"/>
+        <v>12</v>
+      </c>
+      <c r="V17" t="str">
+        <f t="shared" si="9"/>
+        <v>IL</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>81</v>
       </c>
@@ -1803,8 +1983,20 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T18">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V18" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>82</v>
       </c>
@@ -1857,8 +2049,20 @@
         <f t="shared" si="6"/>
         <v>NY</v>
       </c>
+      <c r="T19">
+        <f t="shared" si="7"/>
+        <v>11</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="V19" t="str">
+        <f t="shared" si="9"/>
+        <v>NY</v>
+      </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>87</v>
       </c>
@@ -1911,8 +2115,20 @@
         <f t="shared" si="6"/>
         <v>PA</v>
       </c>
+      <c r="T20">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="V20" t="str">
+        <f t="shared" si="9"/>
+        <v>PA</v>
+      </c>
     </row>
-    <row r="21" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>88</v>
       </c>
@@ -1963,6 +2179,18 @@
       </c>
       <c r="S21" t="str">
         <f t="shared" si="6"/>
+        <v>NY</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="7"/>
+        <v>11</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="V21" t="str">
+        <f t="shared" si="9"/>
         <v>NY</v>
       </c>
     </row>

</xml_diff>